<commit_message>
Update the Charts for the financial ratios.
</commit_message>
<xml_diff>
--- a/03_Charts/VAE/FinancialRatios/XGBoost/BaseModel/Error_Summary.xlsx
+++ b/03_Charts/VAE/FinancialRatios/XGBoost/BaseModel/Error_Summary.xlsx
@@ -20,13 +20,13 @@
     <t xml:space="preserve">Count</t>
   </si>
   <si>
+    <t xml:space="preserve">Median_Return on Assets (ROA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median_Net Debt Ratio</t>
+  </si>
+  <si>
     <t xml:space="preserve">Median_Self-Financing Ratio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Median_Return on Assets (ROA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Median_Net Debt Ratio</t>
   </si>
   <si>
     <t xml:space="preserve">Median_Return on Fixed Assets</t>
@@ -401,22 +401,22 @@
         <v>7</v>
       </c>
       <c r="B2" t="n">
-        <v>119169</v>
+        <v>125115</v>
       </c>
       <c r="C2" t="n">
-        <v>0.239316239316239</v>
+        <v>0.204314036978781</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0487948265726044</v>
+        <v>-0.268050104092045</v>
       </c>
       <c r="E2" t="n">
-        <v>0.439285714285714</v>
+        <v>0.257672962384166</v>
       </c>
       <c r="F2" t="n">
-        <v>0.109350237717908</v>
+        <v>0.156583514125096</v>
       </c>
       <c r="G2" t="n">
-        <v>0.240223463687151</v>
+        <v>0.21965720275054</v>
       </c>
     </row>
     <row r="3">
@@ -424,22 +424,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="n">
-        <v>40861</v>
+        <v>34915</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.0837138508371385</v>
+        <v>-0.944263878788436</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0241935483870968</v>
+        <v>0.920968756252137</v>
       </c>
       <c r="E3" t="n">
-        <v>0.939189189189189</v>
+        <v>-1.00136035550582</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.0447330447330447</v>
+        <v>-0.968666314387297</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0141509433962264</v>
+        <v>-0.670683003564833</v>
       </c>
     </row>
     <row r="4">
@@ -447,22 +447,22 @@
         <v>9</v>
       </c>
       <c r="B4" t="n">
-        <v>241</v>
+        <v>208</v>
       </c>
       <c r="C4" t="n">
-        <v>0.137548530227399</v>
+        <v>-0.0855674357933853</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0277315585135885</v>
+        <v>0.081935835322343</v>
       </c>
       <c r="E4" t="n">
-        <v>0.596485182632667</v>
+        <v>-0.00799816052663417</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0742942050520059</v>
+        <v>-0.106036821317957</v>
       </c>
       <c r="G4" t="n">
-        <v>0.131157270029674</v>
+        <v>-0.00336623411901826</v>
       </c>
     </row>
     <row r="5">
@@ -470,22 +470,22 @@
         <v>10</v>
       </c>
       <c r="B5" t="n">
-        <v>1133</v>
+        <v>1166</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.198019801980198</v>
+        <v>-1.1824998686639</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0646219135802469</v>
+        <v>1.05225686206124</v>
       </c>
       <c r="E5" t="n">
-        <v>1.0088809946714</v>
+        <v>-1.16816871414356</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.197278911564626</v>
+        <v>-1.18458749705223</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0151515151515152</v>
+        <v>-0.642894003289279</v>
       </c>
     </row>
   </sheetData>

</xml_diff>